<commit_message>
FinTrack: add 5 transactions
</commit_message>
<xml_diff>
--- a/data/finance_history.xlsx
+++ b/data/finance_history.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -933,7 +933,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -986,6 +986,146 @@
       </c>
       <c r="F20" t="n">
         <v>13000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Food &amp; Groceries</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Food &amp; Groceries</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Parents / Family</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Parents / Family</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Phone &amp; Internet</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Phone &amp; Internet</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FinTrack: save app state
</commit_message>
<xml_diff>
--- a/data/finance_history.xlsx
+++ b/data/finance_history.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="transactions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="monthly_summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="app_state" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,11 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -52,10 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -989,7 +987,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1017,7 +1015,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1045,7 +1043,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1073,7 +1071,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1101,7 +1099,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1210,4 +1208,32 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>json_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>{"profile": {"name": "Charan", "city": "Bangalore", "employment_type": "Internship", "currency": "INR"}, "income": {"sources": [{"name": "NetApp AI &amp; Digital Experience Intern", "type": "Stipend", "amount": 34567.0, "status": "Active", "id": 1}, {"name": "Freelance / Side Income", "type": "Freelance", "amount": 0.0, "status": "Inactive", "id": 2}, {"name": "Interest / Passive Income", "type": "Rental", "amount": 0.0, "status": "Active", "id": 3}, {"name": NaN, "type": NaN, "amount": NaN, "status": NaN, "id": 4}], "fte_mode": false, "fte_ctc": 1600000, "fte_start_month": 7}, "salary_breakdown": {"enabled": false, "ctc_annual": 1600000, "basic_pct": 40, "hra_pct": 20, "special_allowance_pct": 30, "pf_pct": 12, "professional_tax_monthly": 200, "tax_bracket_pct": 20}, "expenses": {"categories": [{"id": 1, "name": "Rent", "icon": "\ud83c\udfe0", "budget": 15000, "actual": 13000, "group": "Needs"}, {"id": 2, "name": "Food &amp; Groceries", "icon": "\ud83c\udf7d\ufe0f", "budget": 7000, "actual": 7000, "group": "Needs"}, {"id": 3, "name": "Parents / Family", "icon": "\ud83d\udc68\u200d\ud83d\udc69\u200d\ud83d\udc67", "budget": 20000, "actual": 20000, "group": "Needs"}, {"id": 4, "name": "Transport", "icon": "\ud83d\ude8c", "budget": 3000, "actual": 0, "group": "Needs"}, {"id": 5, "name": "Phone &amp; Internet", "icon": "\ud83d\udcf1", "budget": 500, "actual": 500, "group": "Needs"}, {"id": 6, "name": "Health &amp; Medical", "icon": "\ud83c\udfe5", "budget": 1000, "actual": 0, "group": "Needs"}, {"id": 7, "name": "Personal Care", "icon": "\ud83d\udc86", "budget": 1000, "actual": 500, "group": "Wants"}, {"id": 8, "name": "Entertainment", "icon": "\ud83c\udf89", "budget": 1500, "actual": 0, "group": "Wants"}, {"id": 9, "name": "Learning / Courses", "icon": "\ud83d\udcda", "budget": 1000, "actual": 0, "group": "Wants"}, {"id": 10, "name": "Shopping / Misc", "icon": "\ud83d\udecd\ufe0f", "budget": 2000, "actual": 0, "group": "Wants"}], "month_history": {}}, "savings_goals": [{"id": 1, "name": "Emergency Fund", "icon": "\ud83d\udee1\ufe0f", "target": 150000, "saved": 0, "monthly_contribution": 15000, "priority": 1}, {"id": 2, "name": "SIP / Mutual Fund", "icon": "\ud83d\udcc8", "target": 60000, "saved": 0, "monthly_contribution": 5000, "priority": 2}, {"id": 3, "name": "Loan Prepayment Fund", "icon": "\ud83d\udcb0", "target": 100000, "saved": 0, "monthly_contribution": 3000, "priority": 3}, {"id": 4, "name": "Travel Fund", "icon": "\u2708\ufe0f", "target": 30000, "saved": 0, "monthly_contribution": 0, "priority": 4}], "loan": {"account_number": "XXXXXXX5062", "outstanding": 551985, "rate": 9.9, "type": "Education Loan", "status": "Moratorium", "emi_start_month": null, "emi_start_year": null, "tenure_months": 60, "tax_bracket": 20, "rate_history": [{"date": "10/06/2025", "from_rate": 12.65, "to_rate": 10.65}, {"date": "15/06/2025", "from_rate": 10.65, "to_rate": 10.15}, {"date": "15/12/2025", "from_rate": 10.15, "to_rate": 9.9}], "prepayment_amount": 100000, "gold_loan_rate": 9.5}, "net_worth": {"assets": [{"name": "Cash / Savings", "amount": 0}, {"name": "SIP / Mutual Funds", "amount": 0}, {"name": "Gold (grams)", "grams": 0, "rate_per_gram": 9500}, {"name": "Other Assets", "amount": 0}], "liabilities": [{"name": "Education Loan", "amount": 551985}, {"name": "Other Loans", "amount": 0}, {"name": "Credit Card Due", "amount": 0}]}, "ui": {"dismissed_alerts": [], "current_month": "July 2026"}}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
FinTrack: add 1 transactions
</commit_message>
<xml_diff>
--- a/data/finance_history.xlsx
+++ b/data/finance_history.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="transactions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="monthly_summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="app_state" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,9 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1124,6 +1126,34 @@
       </c>
       <c r="F25" t="n">
         <v>500</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Stipend</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NetApp AI &amp; Digital Experience Intern</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>34567</v>
       </c>
     </row>
   </sheetData>
@@ -1208,32 +1238,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>json_data</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>{"profile": {"name": "Charan", "city": "Bangalore", "employment_type": "Internship", "currency": "INR"}, "income": {"sources": [{"name": "NetApp AI &amp; Digital Experience Intern", "type": "Stipend", "amount": 34567.0, "status": "Active", "id": 1}, {"name": "Freelance / Side Income", "type": "Freelance", "amount": 13000.0, "status": "Inactive", "id": 2}, {"name": "Interest / Passive Income", "type": "Rental", "amount": 0.0, "status": "Active", "id": 3}, {"name": NaN, "type": NaN, "amount": NaN, "status": NaN, "id": 4}], "fte_mode": false, "fte_ctc": 1600000, "fte_start_month": 7}, "salary_breakdown": {"enabled": false, "ctc_annual": 1600000, "basic_pct": 40, "hra_pct": 20, "special_allowance_pct": 30, "pf_pct": 12, "professional_tax_monthly": 200, "tax_bracket_pct": 20}, "expenses": {"categories": [{"id": 1, "name": "Rent", "icon": "\ud83c\udfe0", "budget": 15000, "actual": 13000, "group": "Needs"}, {"id": 2, "name": "Food &amp; Groceries", "icon": "\ud83c\udf7d\ufe0f", "budget": 7000, "actual": 7000, "group": "Needs"}, {"id": 3, "name": "Parents / Family", "icon": "\ud83d\udc68\u200d\ud83d\udc69\u200d\ud83d\udc67", "budget": 20000, "actual": 20000, "group": "Needs"}, {"id": 4, "name": "Transport", "icon": "\ud83d\ude8c", "budget": 3000, "actual": 0, "group": "Needs"}, {"id": 5, "name": "Phone &amp; Internet", "icon": "\ud83d\udcf1", "budget": 500, "actual": 500, "group": "Needs"}, {"id": 6, "name": "Health &amp; Medical", "icon": "\ud83c\udfe5", "budget": 1000, "actual": 0, "group": "Needs"}, {"id": 7, "name": "Personal Care", "icon": "\ud83d\udc86", "budget": 1000, "actual": 500, "group": "Wants"}, {"id": 8, "name": "Entertainment", "icon": "\ud83c\udf89", "budget": 1500, "actual": 0, "group": "Wants"}, {"id": 9, "name": "Learning / Courses", "icon": "\ud83d\udcda", "budget": 1000, "actual": 0, "group": "Wants"}, {"id": 10, "name": "Shopping / Misc", "icon": "\ud83d\udecd\ufe0f", "budget": 2000, "actual": 0, "group": "Wants"}], "month_history": {}}, "savings_goals": [{"id": 1, "name": "Emergency Fund", "icon": "\ud83d\udee1\ufe0f", "target": 150000, "saved": 0, "monthly_contribution": 15000, "priority": 1}, {"id": 2, "name": "SIP / Mutual Fund", "icon": "\ud83d\udcc8", "target": 60000, "saved": 0, "monthly_contribution": 5000, "priority": 2}, {"id": 3, "name": "Loan Prepayment Fund", "icon": "\ud83d\udcb0", "target": 100000, "saved": 0, "monthly_contribution": 3000, "priority": 3}, {"id": 4, "name": "Travel Fund", "icon": "\u2708\ufe0f", "target": 30000, "saved": 0, "monthly_contribution": 0, "priority": 4}], "loan": {"account_number": "XXXXXXX5062", "outstanding": 551985, "rate": 9.9, "type": "Education Loan", "status": "Moratorium", "emi_start_month": null, "emi_start_year": null, "tenure_months": 60, "tax_bracket": 20, "rate_history": [{"date": "10/06/2025", "from_rate": 12.65, "to_rate": 10.65}, {"date": "15/06/2025", "from_rate": 10.65, "to_rate": 10.15}, {"date": "15/12/2025", "from_rate": 10.15, "to_rate": 9.9}], "prepayment_amount": 100000, "gold_loan_rate": 9.5}, "net_worth": {"assets": [{"name": "Cash / Savings", "amount": 0}, {"name": "SIP / Mutual Funds", "amount": 0}, {"name": "Gold (grams)", "grams": 0, "rate_per_gram": 9500}, {"name": "Other Assets", "amount": 0}], "liabilities": [{"name": "Education Loan", "amount": 551985}, {"name": "Other Loans", "amount": 0}, {"name": "Credit Card Due", "amount": 0}]}, "ui": {"dismissed_alerts": [], "current_month": "July 2026"}}</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
FinTrack: add 6 transactions
</commit_message>
<xml_diff>
--- a/data/finance_history.xlsx
+++ b/data/finance_history.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="transactions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="monthly_summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="app_state" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,9 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1152,6 +1154,174 @@
       </c>
       <c r="F26" t="n">
         <v>34567</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Food &amp; Groceries</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Food &amp; Groceries</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Phone &amp; Internet</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Phone &amp; Internet</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Shopping / Misc</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Shopping / Misc</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>2045</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -1236,32 +1406,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>json_data</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>{"profile": {"name": "Charan", "city": "Bangalore", "employment_type": "Internship", "currency": "INR"}, "income": {"sources": [{"name": "NetApp AI &amp; Digital Experience Intern", "type": "Stipend", "amount": 34567.0, "status": "Active", "id": 1}, {"name": "Freelance / Side Income", "type": "Freelance", "amount": 13000.0, "status": "Active", "id": 2}, {"name": "Interest / Passive Income", "type": "Rental", "amount": 0.0, "status": "Active", "id": 3}, {"name": "askhfd", "type": NaN, "amount": NaN, "status": NaN, "id": 4}], "fte_mode": false, "fte_ctc": 1600000, "fte_start_month": 7}, "salary_breakdown": {"enabled": false, "ctc_annual": 1600000, "basic_pct": 40, "hra_pct": 20, "special_allowance_pct": 30, "pf_pct": 12, "professional_tax_monthly": 200, "tax_bracket_pct": 20}, "expenses": {"categories": [{"id": 1, "name": "Rent", "icon": "\ud83c\udfe0", "budget": 15000, "actual": 13000, "group": "Needs"}, {"id": 2, "name": "Food &amp; Groceries", "icon": "\ud83c\udf7d\ufe0f", "budget": 7000, "actual": 730, "group": "Needs"}, {"id": 3, "name": "Parents / Family", "icon": "\ud83d\udc68\u200d\ud83d\udc69\u200d\ud83d\udc67", "budget": 20000, "actual": 0, "group": "Needs"}, {"id": 4, "name": "Transport", "icon": "\ud83d\ude8c", "budget": 3000, "actual": 160, "group": "Needs"}, {"id": 5, "name": "Phone &amp; Internet", "icon": "\ud83d\udcf1", "budget": 500, "actual": 300, "group": "Needs"}, {"id": 6, "name": "Health &amp; Medical", "icon": "\ud83c\udfe5", "budget": 1000, "actual": 0, "group": "Needs"}, {"id": 7, "name": "Personal Care", "icon": "\ud83d\udc86", "budget": 1000, "actual": 0, "group": "Wants"}, {"id": 8, "name": "Entertainment", "icon": "\ud83c\udf89", "budget": 1500, "actual": 0, "group": "Wants"}, {"id": 10, "name": "Shopping / Misc", "icon": "\ud83d\udecd\ufe0f", "budget": 2000, "actual": 2045, "group": "Wants"}, {"name": "Groceries", "icon": "\ud83c\udf6a", "budget": 1000, "actual": 285, "group": "Wants", "id": 11}], "month_history": {}}, "savings_goals": [{"id": 1, "name": "Emergency Fund", "icon": "\ud83d\udee1\ufe0f", "target": 150000, "saved": 0, "monthly_contribution": 15000, "priority": 1}, {"id": 2, "name": "SIP / Mutual Fund", "icon": "\ud83d\udcc8", "target": 60000, "saved": 0, "monthly_contribution": 5000, "priority": 2}, {"id": 3, "name": "Loan Prepayment Fund", "icon": "\ud83d\udcb0", "target": 100000, "saved": 0, "monthly_contribution": 3000, "priority": 3}, {"id": 4, "name": "Travel Fund", "icon": "\u2708\ufe0f", "target": 30000, "saved": 0, "monthly_contribution": 0, "priority": 4}], "loan": {"account_number": "XXXXXXX5062", "outstanding": 551985, "rate": 9.9, "type": "Education Loan", "status": "Moratorium", "emi_start_month": null, "emi_start_year": null, "tenure_months": 60, "tax_bracket": 20, "rate_history": [{"date": "10/06/2025", "from_rate": 12.65, "to_rate": 10.65}, {"date": "15/06/2025", "from_rate": 10.65, "to_rate": 10.15}, {"date": "15/12/2025", "from_rate": 10.15, "to_rate": 9.9}], "prepayment_amount": 100000, "gold_loan_rate": 9.5}, "net_worth": {"assets": [{"name": "Cash / Savings", "amount": 0}, {"name": "SIP / Mutual Funds", "amount": 0}, {"name": "Gold (grams)", "grams": 0, "rate_per_gram": 9500}, {"name": "Other Assets", "amount": 0}], "liabilities": [{"name": "Education Loan", "amount": 551985}, {"name": "Other Loans", "amount": 0}, {"name": "Credit Card Due", "amount": 0}]}, "ui": {"dismissed_alerts": [], "current_month": "July 2026"}}</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>